<commit_message>
Log testcase IDs from workbook
</commit_message>
<xml_diff>
--- a/outputs/testcase_workbook/BANG_TESTCASE_THEO_CHUC_NANG_fixed.xlsx
+++ b/outputs/testcase_workbook/BANG_TESTCASE_THEO_CHUC_NANG_fixed.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8400" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Tong hop" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="246">
   <si>
     <t>Bảng Test Case Theo Chức Năng</t>
   </si>
@@ -143,6 +143,9 @@
     <t>Trang hiển thị sản phẩm liên quan đến từ khóa</t>
   </si>
   <si>
+    <t>Medium</t>
+  </si>
+  <si>
     <t>TC_SEARCH_03</t>
   </si>
   <si>
@@ -161,9 +164,6 @@
     <t>Trình duyệt điều hướng sang trang kết quả phù hợp</t>
   </si>
   <si>
-    <t>Medium</t>
-  </si>
-  <si>
     <t>TC_SEARCH_04</t>
   </si>
   <si>
@@ -227,235 +227,238 @@
     <t>Chuỗi rất dài, thao tác paste lặp</t>
   </si>
   <si>
-    <t>Nhập/paste chuỗi lớn vào ô tìm kiếm; tiếp tục paste đến khi không thêm được; thử click sản phẩm (mỗi lần paste 2 triệu ký tự )</t>
+    <t>Nhập/paste chuỗi lớn vào ô tìm kiếm; tiếp tục paste đến khi không thêm được; thử click sản phẩm ( mỗi lần paste 2 triệu ký tự )</t>
   </si>
   <si>
     <t>Hệ thống vẫn phản hồi, ô tìm kiếm không bị trắng/đứng, web giới hạn số kí tự</t>
   </si>
   <si>
+    <t>TC_SEARCH_08</t>
+  </si>
+  <si>
+    <t>Kết quả tìm kiếm nằm đúng vùng kết quả chính</t>
+  </si>
+  <si>
+    <t>Kiểm tra parser không lấy nhầm text ngoài danh sách sản phẩm</t>
+  </si>
+  <si>
+    <t>Tìm kiếm; xác định vùng kết quả chính; trích tên sản phẩm trong vùng đó</t>
+  </si>
+  <si>
+    <t>Danh sách lấy được nằm trong container kết quả chính</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_09</t>
+  </si>
+  <si>
+    <t>Đổi từ khóa cập nhật kết quả</t>
+  </si>
+  <si>
+    <t>Kiểm tra thay đổi keyword làm mới danh sách sản phẩm</t>
+  </si>
+  <si>
+    <t>Hai từ khóa tìm kiếm khác nhau</t>
+  </si>
+  <si>
+    <t>Tìm keyword thứ nhất; lưu kết quả; đổi keyword; tìm lại</t>
+  </si>
+  <si>
+    <t>Kết quả sau khi đổi từ khóa được cập nhật, không giữ danh sách cũ</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_10</t>
+  </si>
+  <si>
+    <t>Tìm kiếm rồi sắp xếp theo giá</t>
+  </si>
+  <si>
+    <t>Kiểm tra kết quả tìm kiếm vẫn liên quan sau khi sort</t>
+  </si>
+  <si>
+    <t>Logitech, sort giá</t>
+  </si>
+  <si>
+    <t>Tìm kiếm keyword; chọn sắp xếp theo giá; đọc tên và giá sản phẩm</t>
+  </si>
+  <si>
+    <t>Sản phẩm vẫn liên quan keyword và giá được sắp đúng</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_11</t>
+  </si>
+  <si>
+    <t>Từ khóa viết thường</t>
+  </si>
+  <si>
+    <t>Kiểm tra tìm kiếm không phân biệt chữ hoa/thường</t>
+  </si>
+  <si>
+    <t>logitech</t>
+  </si>
+  <si>
+    <t>Nhập từ khóa; submit; đọc sản phẩm</t>
+  </si>
+  <si>
+    <t>Kết quả có sản phẩm liên quan Logitech</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_12</t>
+  </si>
+  <si>
+    <t>Từ khóa viết chuẩn</t>
+  </si>
+  <si>
+    <t>Kiểm tra tìm kiếm keyword chuẩn</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_13</t>
+  </si>
+  <si>
+    <t>Từ khóa có khoảng trắng đầu/cuối</t>
+  </si>
+  <si>
+    <t>Kiểm tra hệ thống xử lý trim khoảng trắng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Logitech  </t>
+  </si>
+  <si>
+    <t>Nhập từ khóa có khoảng trắng; submit</t>
+  </si>
+  <si>
+    <t>Kết quả vẫn liên quan Logitech</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_14</t>
+  </si>
+  <si>
+    <t>Từ khóa có ký tự đặc biệt</t>
+  </si>
+  <si>
+    <t>Kiểm tra xử lý ký tự đặc biệt trong keyword</t>
+  </si>
+  <si>
+    <t>Logitech!@#</t>
+  </si>
+  <si>
+    <t>Nhập từ khóa; submit; đọc kết quả</t>
+  </si>
+  <si>
+    <t>Trang không lỗi, kết quả vẫn liên quan hoặc xử lý an toàn</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_15</t>
+  </si>
+  <si>
+    <t>Tìm kiếm typo Logitec</t>
+  </si>
+  <si>
+    <t>Kiểm tra khả năng chịu sai chính tả nhẹ</t>
+  </si>
+  <si>
+    <t>Logitec</t>
+  </si>
+  <si>
+    <t>Nhập keyword typo; submit; đọc kết quả</t>
+  </si>
+  <si>
+    <t>Kết quả vẫn trả về sản phẩm liên quan Logitech</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_16</t>
+  </si>
+  <si>
+    <t>Tìm kiếm typo có khoảng trắng giữa từ</t>
+  </si>
+  <si>
+    <t>Kiểm tra keyword bị tách ký tự vẫn có kết quả liên quan</t>
+  </si>
+  <si>
+    <t>Logit ech</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_17</t>
+  </si>
+  <si>
+    <t>Tìm kiếm typo Logitechk</t>
+  </si>
+  <si>
+    <t>Kiểm tra sai chính tả có thêm ký tự cuối</t>
+  </si>
+  <si>
+    <t>Logitechk</t>
+  </si>
+  <si>
+    <t>Kết quả trả về sản phẩm liên quan Logitech</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_18</t>
+  </si>
+  <si>
+    <t>Tìm kiếm typo Logtech</t>
+  </si>
+  <si>
+    <t>Kiểm tra thiếu ký tự trong keyword</t>
+  </si>
+  <si>
+    <t>Logtech</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_19</t>
+  </si>
+  <si>
+    <t>Tìm kiếm typo có số</t>
+  </si>
+  <si>
+    <t>Kiểm tra keyword lẫn số vẫn xử lý an toàn</t>
+  </si>
+  <si>
+    <t>Logit3ch</t>
+  </si>
+  <si>
+    <t>Kết quả liên quan hoặc trang hiển thị trạng thái hợp lệ</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_20</t>
+  </si>
+  <si>
+    <t>Tìm kiếm không có kết quả</t>
+  </si>
+  <si>
+    <t>Kiểm tra trạng thái no-result</t>
+  </si>
+  <si>
+    <t>nonexistentsku12345</t>
+  </si>
+  <si>
+    <t>Nhập keyword không tồn tại; submit</t>
+  </si>
+  <si>
+    <t>Trang hiển thị trạng thái không có kết quả, không crash</t>
+  </si>
+  <si>
+    <t>TC_SEARCH_21</t>
+  </si>
+  <si>
+    <t>Payload XSS script</t>
+  </si>
+  <si>
+    <t>Kiểm tra payload script không được thực thi trên UI</t>
+  </si>
+  <si>
+    <t>&lt;script&gt;alert(1)&lt;/script&gt;</t>
+  </si>
+  <si>
+    <t>Nhập payload vào ô tìm kiếm; submit; kiểm tra alert và nội dung trang</t>
+  </si>
+  <si>
+    <t>Không xuất hiện alert độc hại, trang xử lý an toàn</t>
+  </si>
+  <si>
     <t>Critical</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_08</t>
-  </si>
-  <si>
-    <t>Kết quả tìm kiếm nằm đúng vùng kết quả chính</t>
-  </si>
-  <si>
-    <t>Kiểm tra parser không lấy nhầm text ngoài danh sách sản phẩm</t>
-  </si>
-  <si>
-    <t>Tìm kiếm; xác định vùng kết quả chính; trích tên sản phẩm trong vùng đó</t>
-  </si>
-  <si>
-    <t>Danh sách lấy được nằm trong container kết quả chính</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_09</t>
-  </si>
-  <si>
-    <t>Đổi từ khóa cập nhật kết quả</t>
-  </si>
-  <si>
-    <t>Kiểm tra thay đổi keyword làm mới danh sách sản phẩm</t>
-  </si>
-  <si>
-    <t>Hai từ khóa tìm kiếm khác nhau</t>
-  </si>
-  <si>
-    <t>Tìm keyword thứ nhất; lưu kết quả; đổi keyword; tìm lại</t>
-  </si>
-  <si>
-    <t>Kết quả sau khi đổi từ khóa được cập nhật, không giữ danh sách cũ</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_10</t>
-  </si>
-  <si>
-    <t>Tìm kiếm rồi sắp xếp theo giá</t>
-  </si>
-  <si>
-    <t>Kiểm tra kết quả tìm kiếm vẫn liên quan sau khi sort</t>
-  </si>
-  <si>
-    <t>Logitech, sort giá</t>
-  </si>
-  <si>
-    <t>Tìm kiếm keyword; chọn sắp xếp theo giá; đọc tên và giá sản phẩm</t>
-  </si>
-  <si>
-    <t>Sản phẩm vẫn liên quan keyword và giá được sắp đúng</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_11</t>
-  </si>
-  <si>
-    <t>Từ khóa viết thường</t>
-  </si>
-  <si>
-    <t>Kiểm tra tìm kiếm không phân biệt chữ hoa/thường</t>
-  </si>
-  <si>
-    <t>logitech</t>
-  </si>
-  <si>
-    <t>Nhập từ khóa; submit; đọc sản phẩm</t>
-  </si>
-  <si>
-    <t>Kết quả có sản phẩm liên quan Logitech</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_12</t>
-  </si>
-  <si>
-    <t>Từ khóa viết chuẩn</t>
-  </si>
-  <si>
-    <t>Kiểm tra tìm kiếm keyword chuẩn</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_13</t>
-  </si>
-  <si>
-    <t>Từ khóa có khoảng trắng đầu/cuối</t>
-  </si>
-  <si>
-    <t>Kiểm tra hệ thống xử lý trim khoảng trắng</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  Logitech  </t>
-  </si>
-  <si>
-    <t>Nhập từ khóa có khoảng trắng; submit</t>
-  </si>
-  <si>
-    <t>Kết quả vẫn liên quan Logitech</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_14</t>
-  </si>
-  <si>
-    <t>Từ khóa có ký tự đặc biệt</t>
-  </si>
-  <si>
-    <t>Kiểm tra xử lý ký tự đặc biệt trong keyword</t>
-  </si>
-  <si>
-    <t>Logitech!@#</t>
-  </si>
-  <si>
-    <t>Nhập từ khóa; submit; đọc kết quả</t>
-  </si>
-  <si>
-    <t>Trang không lỗi, kết quả vẫn liên quan hoặc xử lý an toàn</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_15</t>
-  </si>
-  <si>
-    <t>Tìm kiếm typo Logitec</t>
-  </si>
-  <si>
-    <t>Kiểm tra khả năng chịu sai chính tả nhẹ</t>
-  </si>
-  <si>
-    <t>Logitec</t>
-  </si>
-  <si>
-    <t>Nhập keyword typo; submit; đọc kết quả</t>
-  </si>
-  <si>
-    <t>Kết quả vẫn trả về sản phẩm liên quan Logitech</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_16</t>
-  </si>
-  <si>
-    <t>Tìm kiếm typo có khoảng trắng giữa từ</t>
-  </si>
-  <si>
-    <t>Kiểm tra keyword bị tách ký tự vẫn có kết quả liên quan</t>
-  </si>
-  <si>
-    <t>Logit ech</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_17</t>
-  </si>
-  <si>
-    <t>Tìm kiếm typo Logitechk</t>
-  </si>
-  <si>
-    <t>Kiểm tra sai chính tả có thêm ký tự cuối</t>
-  </si>
-  <si>
-    <t>Logitechk</t>
-  </si>
-  <si>
-    <t>Kết quả trả về sản phẩm liên quan Logitech</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_18</t>
-  </si>
-  <si>
-    <t>Tìm kiếm typo Logtech</t>
-  </si>
-  <si>
-    <t>Kiểm tra thiếu ký tự trong keyword</t>
-  </si>
-  <si>
-    <t>Logtech</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_19</t>
-  </si>
-  <si>
-    <t>Tìm kiếm typo có số</t>
-  </si>
-  <si>
-    <t>Kiểm tra keyword lẫn số vẫn xử lý an toàn</t>
-  </si>
-  <si>
-    <t>Logit3ch</t>
-  </si>
-  <si>
-    <t>Kết quả liên quan hoặc trang hiển thị trạng thái hợp lệ</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_20</t>
-  </si>
-  <si>
-    <t>Tìm kiếm không có kết quả</t>
-  </si>
-  <si>
-    <t>Kiểm tra trạng thái no-result</t>
-  </si>
-  <si>
-    <t>nonexistentsku12345</t>
-  </si>
-  <si>
-    <t>Nhập keyword không tồn tại; submit</t>
-  </si>
-  <si>
-    <t>Trang hiển thị trạng thái không có kết quả, không crash</t>
-  </si>
-  <si>
-    <t>TC_SEARCH_21</t>
-  </si>
-  <si>
-    <t>Payload XSS script</t>
-  </si>
-  <si>
-    <t>Kiểm tra payload script không được thực thi trên UI</t>
-  </si>
-  <si>
-    <t>&lt;script&gt;alert(1)&lt;/script&gt;</t>
-  </si>
-  <si>
-    <t>Nhập payload vào ô tìm kiếm; submit; kiểm tra alert và nội dung trang</t>
-  </si>
-  <si>
-    <t>Không xuất hiện alert độc hại, trang xử lý an toàn</t>
   </si>
   <si>
     <t>TC_SEARCH_22</t>
@@ -807,7 +810,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF991B1B"/>
+      <color rgb="FF9A3412"/>
       <name val="Carlito"/>
       <charset val="134"/>
     </font>
@@ -821,7 +824,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF9A3412"/>
+      <color rgb="FF991B1B"/>
       <name val="Carlito"/>
       <charset val="134"/>
     </font>
@@ -977,7 +980,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1004,19 +1007,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFEDD5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF9C3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFEE2E2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF9C3"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEDD5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1367,7 +1376,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1391,16 +1400,16 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1409,89 +1418,89 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1511,7 +1520,10 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2171,7 +2183,7 @@
       <c r="F5" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="5" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2194,31 +2206,31 @@
       <c r="F6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="7" t="s">
-        <v>30</v>
+      <c r="G6" s="6" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="7" ht="58.5" customHeight="1" spans="1:7">
       <c r="A7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" ht="58.5" customHeight="1" spans="1:7">
@@ -2240,8 +2252,8 @@
       <c r="F8" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G8" s="7" t="s">
-        <v>30</v>
+      <c r="G8" s="6" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="9" ht="58.5" customHeight="1" spans="1:7">
@@ -2264,7 +2276,7 @@
         <v>54</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" ht="58.5" customHeight="1" spans="1:7">
@@ -2287,7 +2299,7 @@
         <v>60</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" ht="58.5" customHeight="1" spans="1:7">
@@ -2310,99 +2322,99 @@
         <v>66</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>67</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" ht="58.5" customHeight="1" spans="1:7">
       <c r="A12" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>70</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>27</v>
       </c>
       <c r="E12" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>30</v>
+      <c r="G12" s="6" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="13" ht="58.5" customHeight="1" spans="1:7">
       <c r="A13" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B13" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="C13" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="E13" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="F13" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="G13" s="7" t="s">
+      <c r="G13" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="14" ht="58.5" customHeight="1" spans="1:7">
       <c r="A14" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B14" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="C14" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="E14" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="F14" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="F14" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="15" ht="58.5" customHeight="1" spans="1:7">
       <c r="A15" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="E15" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="4" t="s">
+      <c r="F15" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="F15" s="4" t="s">
+      <c r="G15" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="16" ht="58.5" customHeight="1" spans="1:7">
@@ -2419,13 +2431,13 @@
         <v>27</v>
       </c>
       <c r="E16" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="F16" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="G16" s="7" t="s">
         <v>90</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="17" ht="58.5" customHeight="1" spans="1:7">
@@ -2447,8 +2459,8 @@
       <c r="F17" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="G17" s="6" t="s">
-        <v>43</v>
+      <c r="G17" s="7" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="18" ht="58.5" customHeight="1" spans="1:7">
@@ -2471,7 +2483,7 @@
         <v>105</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" ht="58.5" customHeight="1" spans="1:7">
@@ -2493,8 +2505,8 @@
       <c r="F19" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="G19" s="6" t="s">
-        <v>43</v>
+      <c r="G19" s="7" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="20" ht="58.5" customHeight="1" spans="1:7">
@@ -2516,8 +2528,8 @@
       <c r="F20" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="G20" s="6" t="s">
-        <v>43</v>
+      <c r="G20" s="7" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="21" ht="58.5" customHeight="1" spans="1:7">
@@ -2539,8 +2551,8 @@
       <c r="F21" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="G21" s="6" t="s">
-        <v>43</v>
+      <c r="G21" s="7" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="22" ht="58.5" customHeight="1" spans="1:7">
@@ -2562,8 +2574,8 @@
       <c r="F22" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="G22" s="6" t="s">
-        <v>43</v>
+      <c r="G22" s="7" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="23" ht="58.5" customHeight="1" spans="1:7">
@@ -2585,8 +2597,8 @@
       <c r="F23" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="G23" s="6" t="s">
-        <v>43</v>
+      <c r="G23" s="7" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="24" ht="58.5" customHeight="1" spans="1:7">
@@ -2608,7 +2620,7 @@
       <c r="F24" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="G24" s="7" t="s">
+      <c r="G24" s="5" t="s">
         <v>30</v>
       </c>
     </row>
@@ -2631,192 +2643,192 @@
       <c r="F25" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="G25" s="5" t="s">
-        <v>67</v>
+      <c r="G25" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="26" ht="58.5" customHeight="1" spans="1:7">
       <c r="A26" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="G26" s="8" t="s">
         <v>142</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="D26" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="F26" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="27" ht="58.5" customHeight="1" spans="1:7">
       <c r="A27" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>67</v>
+        <v>154</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="28" ht="58.5" customHeight="1" spans="1:7">
       <c r="A28" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>67</v>
+        <v>160</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="29" ht="58.5" customHeight="1" spans="1:7">
       <c r="A29" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>67</v>
+        <v>165</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="30" ht="58.5" customHeight="1" spans="1:7">
       <c r="A30" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>67</v>
+        <v>170</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="31" ht="58.5" customHeight="1" spans="1:7">
       <c r="A31" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="G31" s="5" t="s">
-        <v>67</v>
+        <v>175</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="32" ht="58.5" customHeight="1" spans="1:7">
       <c r="A32" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="G32" s="5" t="s">
-        <v>67</v>
+        <v>180</v>
+      </c>
+      <c r="G32" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="33" ht="58.5" customHeight="1" spans="1:7">
       <c r="A33" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>67</v>
+        <v>185</v>
+      </c>
+      <c r="G33" s="8" t="s">
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -2845,25 +2857,25 @@
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" ht="21" customHeight="1" spans="1:7">
@@ -2914,139 +2926,139 @@
     </row>
     <row r="5" ht="58.5" customHeight="1" spans="1:7">
       <c r="A5" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="G5" s="7" t="s">
+        <v>192</v>
+      </c>
+      <c r="G5" s="5" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="6" ht="58.5" customHeight="1" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="G6" s="7" t="s">
-        <v>30</v>
+        <v>197</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="7" ht="58.5" customHeight="1" spans="1:7">
       <c r="A7" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" ht="58.5" customHeight="1" spans="1:7">
       <c r="A8" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>30</v>
+        <v>209</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="9" ht="58.5" customHeight="1" spans="1:7">
       <c r="A9" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>30</v>
+        <v>214</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="10" ht="58.5" customHeight="1" spans="1:7">
       <c r="A10" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="G10" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>30</v>
       </c>
     </row>
@@ -3076,25 +3088,25 @@
   <sheetData>
     <row r="1" ht="25.5" customHeight="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="2" ht="21" customHeight="1" spans="1:7">
@@ -3145,94 +3157,94 @@
     </row>
     <row r="5" ht="58.5" customHeight="1" spans="1:7">
       <c r="A5" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>67</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" ht="58.5" customHeight="1" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" ht="58.5" customHeight="1" spans="1:7">
       <c r="A7" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>30</v>
+        <v>239</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="8" ht="58.5" customHeight="1" spans="1:7">
       <c r="A8" s="4" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>30</v>
+        <v>245</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>